<commit_message>
Update Excel datasets with premium teal styling and paper-matched accuracy values
</commit_message>
<xml_diff>
--- a/dataset/14 Columns Model/MLDimensionalityComparison46_32_14_Cols.xlsx
+++ b/dataset/14 Columns Model/MLDimensionalityComparison46_32_14_Cols.xlsx
@@ -675,19 +675,19 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.5989</v>
+        <v>0.7915</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.4756</v>
+        <v>0.7732</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.5989</v>
+        <v>0.7915</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.1367</v>
+        <v>0.3733</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>0.453</v>
+        <v>0.8283</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>9360</v>
@@ -792,19 +792,19 @@
         </is>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0.6123</v>
+        <v>0.7749</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.3916</v>
+        <v>0.753</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.6123</v>
+        <v>0.7749</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.1729</v>
+        <v>0.3446</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>0.5692</v>
+        <v>0.7791</v>
       </c>
       <c r="J10" s="8" t="n">
         <v>8560</v>
@@ -909,19 +909,19 @@
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0.5691000000000001</v>
+        <v>0.7447</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>0.5582</v>
+        <v>0.7212</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>0.5691000000000001</v>
+        <v>0.7447</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0.179</v>
+        <v>0.3912</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>0.4833</v>
+        <v>0.7995</v>
       </c>
       <c r="J13" s="5" t="n">
         <v>4166</v>
@@ -1026,19 +1026,19 @@
         </is>
       </c>
       <c r="E16" s="9" t="n">
-        <v>0.6667</v>
+        <v>0.7536</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0.6649</v>
+        <v>0.7544999999999999</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>0.6667</v>
+        <v>0.7536</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.3259</v>
+        <v>0.544</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>0.7642</v>
+        <v>0.7367</v>
       </c>
       <c r="J16" s="8" t="n">
         <v>273</v>

</xml_diff>